<commit_message>
feat: add custom crawlers for new sources
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R70c756cd7dcc4fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7149f6c19740479c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1060,11 +1060,11 @@
           <x:t xml:space="preserve">光伏技术、产业、市场、政策综合资讯</x:t>
         </x:is>
       </x:c>
-      <x:c r="G19" s="1" t="n"/>
-      <x:c r="H19" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://news.solarbe.com/technology</x:t>
-        </x:is>
+      <x:c r="G19" s="1" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取光伏要闻列表。</x:v>
+      </x:c>
+      <x:c r="H19" s="1" t="str">
+        <x:v>https://news.solarbe.com/yaowen</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2217,6 +2217,266 @@
         <x:is>
           <x:t xml:space="preserve">https://www.ithome.com/</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>光伏测试网</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>光伏</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>光伏要闻</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>光伏产业、项目、企业与技术新闻；读取指定 Discuz 门户栏目。</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；仅采集 portal.php?mod=view&amp;aid=... 新闻详情。</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>http://www.testpv.com/portal.php?mod=list&amp;catid=20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>国际能源网</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>综合能源媒体</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>综合新能源</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>宏观/国内政策/国际政策</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>能源行业宏观动态及国内、国际能源政策。</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取 news、policy/intl、policy/china 三个栏目。</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>https://www.in-en.com/article/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>中国能源网</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>综合能源媒体</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>综合新能源</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>能源经济</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>能源经济、政策与产业运行新闻。</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>来自 sources II.xlsx；首页会跳转会话页，定制读取无需登录的 energy-economy 公开栏目。</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>https://www.china5e.com/news/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>我爱电车网</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>新能源汽车/储能</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>新能源汽车、动力电池、储能项目与企业动态。</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取首页新闻卡片并过滤侧栏旧闻。</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>https://www.xevcar.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>北极星储能网</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>储能</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>要闻/独家/市场</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>储能政策、市场、项目、技术和企业动态。</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取要闻、独家、市场三个栏目。</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>https://chuneng.bjx.com.cn/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>INSIDEEVs</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>电动汽车</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>全球电动汽车、电池、充电与电动交通产业新闻。</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>来自 sources II.xlsx；RSS: https://insideevs.com/rss/news/all/；网页列表 403 时以官方 News RSS 为主。</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>https://insideevs.com/news/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>EnergyTrend储能</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>储能</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>储能/电池/光伏</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>集邦新能源网的储能、电池与新能源产业新闻。</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取 news 页面，排除 RSS 中的价格与研究栏目。</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>https://www.energytrend.cn/news/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>NE时代</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>新能源汽车/智能汽车</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>新能源汽车、电池、电驱、智能驾驶与供应链资讯。</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取“全部”文章列表 /web/article/{id}。</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>https://www.ne-time.cn/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>电池网</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>国内/国际/企业新闻</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>电池新能源产业链、项目、技术、政策与企业动态。</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取国内、国际、企业新闻三个栏目。</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>https://www.itdcw.com/news/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>X-MOL</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>科研资讯平台</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>化学/材料</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>化学、材料、纳米、高分子及相关科研资讯。</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>来自 sources II.xlsx；需账号登录；公开化学资讯入口会跳转登录页，未配置授权凭据时默认跳过。</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>https://www.x-mol.com/news/chem</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: repair and extend news channels
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7149f6c19740479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Reacda9717a7b4cb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,10 +38,16 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="4">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -481,46 +487,30 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">batteries news</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">垂直领域媒体</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">电池</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">实时</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">综合类电池新闻网站</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">公司无法访问</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H5" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://batteriesnews.com/</x:t>
-        </x:is>
+    <x:row r="5" ht="108" customHeight="1">
+      <x:c r="A5" s="1" t="str">
+        <x:v>Batteries News</x:v>
+      </x:c>
+      <x:c r="B5" s="1" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="str">
+        <x:v>电池</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>综合电池新闻/市场情报</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="str">
+        <x:v>每日采集首页 Latest 板块的电池行业新闻与市场情报。</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="str">
+        <x:v>HTML 抓取；限定标题为 Latest 的 gridlove-module；读取 article.gridlove-post；跟随 Load More 的 /page/N/ 分页；详情正文限定 .entry-content。</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="str">
+        <x:v>https://batteriesnews.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="27.600000381469727" customHeight="1">
@@ -907,46 +897,30 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16" ht="55.20000076293945" customHeight="1">
-      <x:c r="A16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">interesting engineering</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">垂直领域媒体</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">综合科技</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">实时</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">涉及能源、AI/机器人、太空、军事、交通（陆海空）、健康、文化（科学伦理、人类起源发展及个人隐私）、及其他科学创新（未作细分划分）；整体信息更偏向前沿技术开发研究，内容为原文转载/原文加工转述，标题较为夸张存在渲染性表达，选录内容仍需进一步组织和挖掘</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">来自 news-search-main；RSS: https://interestingengineering.com/feed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H16" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://interestingengineering.com/news</x:t>
-        </x:is>
+    <x:row r="16" ht="108" customHeight="1">
+      <x:c r="A16" s="1" t="str">
+        <x:v>interesting engineering</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D16" s="1" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str">
+        <x:v>涉及能源、AI/机器人、太空、军事、交通（陆海空）、健康、文化（科学伦理、人类起源发展及个人隐私）、及其他科学创新（未作细分划分）；整体信息更偏向前沿技术开发研究，内容为原文转载/原文加工转述，标题较为夸张存在渲染性表达，选录内容仍需进一步组织和挖掘</x:v>
+      </x:c>
+      <x:c r="G16" s="2" t="str">
+        <x:v>定制抓取：https://interestingengineering.com/news；按日期分组读取新闻卡片，跟随 aria-label=Go to next page 的 /news/page/N 分页；官方 RSS: https://interestingengineering.com/feed 的 content:encoded 全文优先，RSS 未覆盖时仅读取详情页 .body-content 公开预览；不绕过订阅墙。</x:v>
+      </x:c>
+      <x:c r="H16" s="2" t="str">
+        <x:v>https://interestingengineering.com/news</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="27.600000381469727" customHeight="1">
@@ -1493,40 +1467,30 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">pv magazine C&amp;I PV</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B31" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">垂直领域媒体</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C31" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">光伏</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D31" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">工商业光伏</x:t>
-        </x:is>
+    <x:row r="31" ht="108" customHeight="1">
+      <x:c r="A31" s="1" t="str">
+        <x:v>pv magazine C&amp;I PV</x:v>
+      </x:c>
+      <x:c r="B31" s="1" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C31" s="1" t="str">
+        <x:v>光伏</x:v>
+      </x:c>
+      <x:c r="D31" s="1" t="str">
+        <x:v>工商业光伏</x:v>
       </x:c>
       <x:c r="E31" s="1" t="str">
         <x:v>工作日</x:v>
       </x:c>
-      <x:c r="F31" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">pv magazine 工商业光伏安装与应用频道。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G31" s="1" t="str">
-        <x:v>HTML 抓取；已迁移到 pv magazine 官方 Commercial &amp; industrial 标签页；原分类 RSS 已失效。</x:v>
-      </x:c>
-      <x:c r="H31" s="1" t="str">
-        <x:v>https://www.pv-magazine.com/tag/commercial-industrial/</x:v>
+      <x:c r="F31" s="2" t="str">
+        <x:v>pv magazine 工商业光伏安装与应用频道。</x:v>
+      </x:c>
+      <x:c r="G31" s="2" t="str">
+        <x:v>HTML 抓取；用户指定从 pvmagazine-article-feed 的 __container 边界后读取 __inner，排除页面上半部分 Post Grid；跟随底部 Next 分页；详情正文限定 .pvmagazine-post-content .entry-content。</x:v>
+      </x:c>
+      <x:c r="H31" s="2" t="str">
+        <x:v>https://www.pv-magazine.com/latest-news/</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2245,7 +2209,7 @@
         <x:v>http://www.testpv.com/portal.php?mod=list&amp;catid=20</x:v>
       </x:c>
     </x:row>
-    <x:row r="50">
+    <x:row r="50" ht="108" customHeight="1">
       <x:c r="A50" t="str">
         <x:v>国际能源网</x:v>
       </x:c>
@@ -2261,17 +2225,17 @@
       <x:c r="E50" t="str">
         <x:v>实时</x:v>
       </x:c>
-      <x:c r="F50" t="str">
+      <x:c r="F50" s="3" t="str">
         <x:v>能源行业宏观动态及国内、国际能源政策。</x:v>
       </x:c>
-      <x:c r="G50" t="str">
-        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取 news、policy/intl、policy/china 三个栏目。</x:v>
-      </x:c>
-      <x:c r="H50" t="str">
+      <x:c r="G50" s="3" t="str">
+        <x:v>停止直接抓取网页；改由 RIOnews API/每日 Excel 导入，仅接收“发布媒体”以“国际能源网_”开头的记录（宏观新闻栏目）；本地通过 RIONEWS_DAILY_DIR 配置，GitHub Actions 使用 Secrets 拉取。</x:v>
+      </x:c>
+      <x:c r="H50" s="3" t="str">
         <x:v>https://www.in-en.com/article/</x:v>
       </x:c>
     </x:row>
-    <x:row r="51">
+    <x:row r="51" ht="108" customHeight="1">
       <x:c r="A51" t="str">
         <x:v>中国能源网</x:v>
       </x:c>
@@ -2287,17 +2251,17 @@
       <x:c r="E51" t="str">
         <x:v>工作日</x:v>
       </x:c>
-      <x:c r="F51" t="str">
+      <x:c r="F51" s="3" t="str">
         <x:v>能源经济、政策与产业运行新闻。</x:v>
       </x:c>
-      <x:c r="G51" t="str">
-        <x:v>来自 sources II.xlsx；首页会跳转会话页，定制读取无需登录的 energy-economy 公开栏目。</x:v>
-      </x:c>
-      <x:c r="H51" t="str">
+      <x:c r="G51" s="3" t="str">
+        <x:v>停止直接抓取中国能源网页面；改由 RIOnews API/每日 Excel 导入，仅接收“发布媒体”以“中国能源网_”开头的记录（新能源、节能低碳）；本地通过 RIONEWS_DAILY_DIR 配置，GitHub Actions 使用 Secrets 拉取。</x:v>
+      </x:c>
+      <x:c r="H51" s="3" t="str">
         <x:v>https://www.china5e.com/news/</x:v>
       </x:c>
     </x:row>
-    <x:row r="52">
+    <x:row r="52" ht="108" customHeight="1">
       <x:c r="A52" t="str">
         <x:v>我爱电车网</x:v>
       </x:c>
@@ -2313,13 +2277,13 @@
       <x:c r="E52" t="str">
         <x:v>实时</x:v>
       </x:c>
-      <x:c r="F52" t="str">
+      <x:c r="F52" s="3" t="str">
         <x:v>新能源汽车、动力电池、储能项目与企业动态。</x:v>
       </x:c>
-      <x:c r="G52" t="str">
-        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取首页新闻卡片并过滤侧栏旧闻。</x:v>
-      </x:c>
-      <x:c r="H52" t="str">
+      <x:c r="G52" s="3" t="str">
+        <x:v>停止直接抓取网页；改由 RIOnews API/每日 Excel 导入，仅接收“发布媒体”以“我爱电车网_”开头的记录（首页新闻）；本地通过 RIONEWS_DAILY_DIR 配置，GitHub Actions 使用 Secrets 拉取。</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="str">
         <x:v>https://www.xevcar.com/</x:v>
       </x:c>
     </x:row>
@@ -2375,7 +2339,7 @@
         <x:v>https://insideevs.com/news/</x:v>
       </x:c>
     </x:row>
-    <x:row r="55">
+    <x:row r="55" ht="108" customHeight="1">
       <x:c r="A55" t="str">
         <x:v>EnergyTrend储能</x:v>
       </x:c>
@@ -2391,13 +2355,13 @@
       <x:c r="E55" t="str">
         <x:v>工作日</x:v>
       </x:c>
-      <x:c r="F55" t="str">
+      <x:c r="F55" s="3" t="str">
         <x:v>集邦新能源网的储能、电池与新能源产业新闻。</x:v>
       </x:c>
-      <x:c r="G55" t="str">
-        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取 news 页面，排除 RSS 中的价格与研究栏目。</x:v>
-      </x:c>
-      <x:c r="H55" t="str">
+      <x:c r="G55" s="3" t="str">
+        <x:v>RSS: https://www.energytrend.cn/rss.xml；仅接受 /news/YYYYMMDD-ID.html 新闻链接，排除 pricequotes 价格和 research 研究栏目；RSS 无摘要时读取详情正文。</x:v>
+      </x:c>
+      <x:c r="H55" s="3" t="str">
         <x:v>https://www.energytrend.cn/news/</x:v>
       </x:c>
     </x:row>
@@ -2427,7 +2391,7 @@
         <x:v>https://www.ne-time.cn/</x:v>
       </x:c>
     </x:row>
-    <x:row r="57">
+    <x:row r="57" ht="108" customHeight="1">
       <x:c r="A57" t="str">
         <x:v>电池网</x:v>
       </x:c>
@@ -2443,13 +2407,13 @@
       <x:c r="E57" t="str">
         <x:v>实时</x:v>
       </x:c>
-      <x:c r="F57" t="str">
+      <x:c r="F57" s="3" t="str">
         <x:v>电池新能源产业链、项目、技术、政策与企业动态。</x:v>
       </x:c>
-      <x:c r="G57" t="str">
-        <x:v>来自 sources II.xlsx；HTML 抓取；定制读取国内、国际、企业新闻三个栏目。</x:v>
-      </x:c>
-      <x:c r="H57" t="str">
+      <x:c r="G57" s="3" t="str">
+        <x:v>停止直接抓取网页；改由 RIOnews API/每日 Excel 导入，仅接收“发布媒体”以“电池网_”开头的记录（国内、企业等新闻栏目）；本地通过 RIONEWS_DAILY_DIR 配置，GitHub Actions 使用 Secrets 拉取。</x:v>
+      </x:c>
+      <x:c r="H57" s="3" t="str">
         <x:v>https://www.itdcw.com/news/</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add UIED source discovery and stabilize perovskite feed
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1f29be1528a648f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra105a588e51e4be0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -997,7 +997,7 @@
         </x:is>
       </x:c>
       <x:c r="G18" s="1" t="str">
-        <x:v>HTML 抓取；直接读取 Perovskite-Info 公开列表与详情页；原 Google News RSS 受 robots.txt 限制，已停用。</x:v>
+        <x:v>RSS: https://www.perovskite-info.com/rss.xml；官方 RSS 主入口；专用 HTML 列表作为备用；不再使用 Google News RSS。</x:v>
       </x:c>
       <x:c r="H18" s="1" t="inlineStr">
         <x:is>
@@ -2172,10 +2172,8 @@
           <x:t xml:space="preserve">IT之家科技资讯 RSS，覆盖科技、数码、互联网、软硬件与行业动态。</x:t>
         </x:is>
       </x:c>
-      <x:c r="G48" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RSS: https://www.ithome.com/rss/</x:t>
-        </x:is>
+      <x:c r="G48" s="1" t="str">
+        <x:v>RSS: https://www.ithome.com/rss/；聚合备用RSS: https://uiedtool.com/rss-proxy/rss；发现平台: https://uiedtool.com/tools/ai-news。</x:v>
       </x:c>
       <x:c r="H48" s="1" t="inlineStr">
         <x:is>
@@ -2467,6 +2465,110 @@
       </x:c>
       <x:c r="H59" t="str">
         <x:v>https://www.datacenterknowledge.com/latest-news</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>36氪</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>综合科技媒体</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>科技创业/产业</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>科技、创业、投融资、互联网及产业创新资讯。</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/36kr-proxy/feed；聚合入口不可用时回退原站列表。</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>https://36kr.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>少数派</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>综合科技媒体</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>数字产品/效率工具</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>数字产品、软件服务、效率工具及科技生活资讯。</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/sspai-proxy/feed；保留原文链接并按少数派归档。</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>https://sspai.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>机器之心</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>人工智能</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>人工智能研究、产品、企业、算力及产业应用资讯。</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/jqzx-proxy/rss；聚合入口不可用时回退原站列表。</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>https://www.jiqizhixin.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>量子位</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>垂直领域媒体</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>人工智能</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>实时</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>人工智能、机器人、模型、芯片及科技企业资讯。</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/quantumu-proxy/feed；聚合入口不可用时回退原站列表。</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>https://www.qbitai.com/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Avoid inactive UIED proxy channels
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra105a588e51e4be0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Raf54fa3dc6b8445a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2469,7 +2469,7 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" t="str">
-        <x:v>36氪</x:v>
+        <x:v>少数派</x:v>
       </x:c>
       <x:c r="B60" t="str">
         <x:v>综合科技媒体</x:v>
@@ -2478,98 +2478,66 @@
         <x:v>综合科技</x:v>
       </x:c>
       <x:c r="D60" t="str">
-        <x:v>科技创业/产业</x:v>
+        <x:v>数字产品/效率工具</x:v>
       </x:c>
       <x:c r="E60" t="str">
         <x:v>实时</x:v>
       </x:c>
       <x:c r="F60" t="str">
-        <x:v>科技、创业、投融资、互联网及产业创新资讯。</x:v>
+        <x:v>数字产品、软件服务、效率工具及科技生活资讯。</x:v>
       </x:c>
       <x:c r="G60" t="str">
-        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/36kr-proxy/feed；聚合入口不可用时回退原站列表。</x:v>
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/sspai-proxy/feed；保留原文链接并按少数派归档。</x:v>
       </x:c>
       <x:c r="H60" t="str">
-        <x:v>https://36kr.com/</x:v>
+        <x:v>https://sspai.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" t="str">
-        <x:v>少数派</x:v>
+        <x:v>量子位</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>综合科技媒体</x:v>
+        <x:v>垂直领域媒体</x:v>
       </x:c>
       <x:c r="C61" t="str">
         <x:v>综合科技</x:v>
       </x:c>
       <x:c r="D61" t="str">
-        <x:v>数字产品/效率工具</x:v>
+        <x:v>人工智能</x:v>
       </x:c>
       <x:c r="E61" t="str">
         <x:v>实时</x:v>
       </x:c>
       <x:c r="F61" t="str">
-        <x:v>数字产品、软件服务、效率工具及科技生活资讯。</x:v>
+        <x:v>人工智能、机器人、模型、芯片及科技企业资讯。</x:v>
       </x:c>
       <x:c r="G61" t="str">
-        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/sspai-proxy/feed；保留原文链接并按少数派归档。</x:v>
+        <x:v>发现平台: https://uiedtool.com/tools/ai-news；当前聚合代理返回 403，暂不作为程序入口；直接抓取量子位原站列表并保留原始来源名。</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>https://sspai.com/</x:v>
+        <x:v>https://www.qbitai.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" t="str">
-        <x:v>机器之心</x:v>
-      </x:c>
-      <x:c r="B62" t="str">
-        <x:v>垂直领域媒体</x:v>
-      </x:c>
-      <x:c r="C62" t="str">
-        <x:v>综合科技</x:v>
-      </x:c>
-      <x:c r="D62" t="str">
-        <x:v>人工智能</x:v>
-      </x:c>
-      <x:c r="E62" t="str">
-        <x:v>实时</x:v>
-      </x:c>
-      <x:c r="F62" t="str">
-        <x:v>人工智能研究、产品、企业、算力及产业应用资讯。</x:v>
-      </x:c>
-      <x:c r="G62" t="str">
-        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/jqzx-proxy/rss；聚合入口不可用时回退原站列表。</x:v>
-      </x:c>
-      <x:c r="H62" t="str">
-        <x:v>https://www.jiqizhixin.com/</x:v>
-      </x:c>
+      <x:c r="A62"/>
+      <x:c r="B62"/>
+      <x:c r="C62"/>
+      <x:c r="D62"/>
+      <x:c r="E62"/>
+      <x:c r="F62"/>
+      <x:c r="G62"/>
+      <x:c r="H62"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" t="str">
-        <x:v>量子位</x:v>
-      </x:c>
-      <x:c r="B63" t="str">
-        <x:v>垂直领域媒体</x:v>
-      </x:c>
-      <x:c r="C63" t="str">
-        <x:v>综合科技</x:v>
-      </x:c>
-      <x:c r="D63" t="str">
-        <x:v>人工智能</x:v>
-      </x:c>
-      <x:c r="E63" t="str">
-        <x:v>实时</x:v>
-      </x:c>
-      <x:c r="F63" t="str">
-        <x:v>人工智能、机器人、模型、芯片及科技企业资讯。</x:v>
-      </x:c>
-      <x:c r="G63" t="str">
-        <x:v>发现平台: https://uiedtool.com/tools/ai-news；聚合RSS: https://uiedtool.com/quantumu-proxy/feed；聚合入口不可用时回退原站列表。</x:v>
-      </x:c>
-      <x:c r="H63" t="str">
-        <x:v>https://www.qbitai.com/</x:v>
-      </x:c>
+      <x:c r="A63"/>
+      <x:c r="B63"/>
+      <x:c r="C63"/>
+      <x:c r="D63"/>
+      <x:c r="E63"/>
+      <x:c r="F63"/>
+      <x:c r="G63"/>
+      <x:c r="H63"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add local The Information daily ingest
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Raf54fa3dc6b8445a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R05ce3208e1a04337"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1219,7 +1219,7 @@
         </x:is>
       </x:c>
       <x:c r="G24" s="1" t="str">
-        <x:v>RSS: https://www.theinformation.com/feed；正文受订阅限制时使用 RSS 中公开摘要，不绕过付费墙。</x:v>
+        <x:v>RSS: https://www.theinformation.com/feed；订阅全文由本地 Windows 计划任务通过认证 Feed 抓取，日分片上传 the-information-inbox 分支后由 GitHub Actions 幂等汇总；云端每日主任务跳过直接抓取。</x:v>
       </x:c>
       <x:c r="H24" s="1" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
Fix The Information public RSS ingest
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R05ce3208e1a04337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R05211df233594d82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1219,7 +1219,7 @@
         </x:is>
       </x:c>
       <x:c r="G24" s="1" t="str">
-        <x:v>RSS: https://www.theinformation.com/feed；订阅全文由本地 Windows 计划任务通过认证 Feed 抓取，日分片上传 the-information-inbox 分支后由 GitHub Actions 幂等汇总；云端每日主任务跳过直接抓取。</x:v>
+        <x:v>RSS: https://www.theinformation.com/feed；本地 Windows 计划任务仅抓取公开 RSS 标题、日期、原文链接和摘要；直接访问被 Cloudflare 拦截时使用 Feedly 标准公开阅读器接口；日分片上传 the-information-inbox 分支后由 GitHub Actions 幂等汇总；不读取订阅页或认证凭据。</x:v>
       </x:c>
       <x:c r="H24" s="1" t="inlineStr">
         <x:is>

</xml_diff>